<commit_message>
Update implementation status tracker for 0.3.1
</commit_message>
<xml_diff>
--- a/Events.xlsx
+++ b/Events.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="111">
   <si>
     <t xml:space="preserve">Event Name</t>
   </si>
@@ -100,7 +100,7 @@
     <t xml:space="preserve">TipGoalUpdated</t>
   </si>
   <si>
-    <t xml:space="preserve">{"title":"Flast Tits"</t>
+    <t xml:space="preserve">{"title":"Flash Tits"</t>
   </si>
   <si>
     <t xml:space="preserve">"amount":10000}</t>
@@ -313,22 +313,37 @@
     <t xml:space="preserve">StreamEnding</t>
   </si>
   <si>
+    <t xml:space="preserve">Implemented – Tested OK</t>
+  </si>
+  <si>
     <t xml:space="preserve">StreamModeUpdated</t>
   </si>
   <si>
+    <t xml:space="preserve">Implemented – should work</t>
+  </si>
+  <si>
     <t xml:space="preserve">StreamResuming</t>
   </si>
   <si>
+    <t xml:space="preserve">Implemented – might work</t>
+  </si>
+  <si>
     <t xml:space="preserve">Started</t>
   </si>
   <si>
     <t xml:space="preserve">{"who":”breakfast”}</t>
   </si>
   <si>
+    <t xml:space="preserve">Implemented – known broken</t>
+  </si>
+  <si>
     <t xml:space="preserve">DeviceConnected</t>
   </si>
   <si>
     <t xml:space="preserve">{}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not Implemented</t>
   </si>
   <si>
     <t xml:space="preserve">DeviceDisconnected</t>
@@ -347,11 +362,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -368,8 +384,15 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -385,13 +408,25 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FF993300"/>
+        <bgColor rgb="FFFF4000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF81D41A"/>
         <bgColor rgb="FF969696"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF008000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF4000"/>
+        <bgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -429,24 +464,40 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -459,39 +510,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF81D41A"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -539,11 +557,11 @@
       <rgbColor rgb="FF81D41A"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FFFF4000"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF00A933"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
@@ -674,526 +692,569 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.93"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="C1" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="D1" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="E1" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" s="3" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>4</v>
       </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="6" t="s">
         <v>21</v>
       </c>
+      <c r="F7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="6" t="s">
         <v>41</v>
       </c>
+      <c r="F13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="4" t="s">
+      <c r="B14" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="B15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C16" s="4" t="s">
+      <c r="B16" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="B17" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="4" t="s">
         <v>52</v>
       </c>
+      <c r="F17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="2" t="s">
+      <c r="B18" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="2"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="B19" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="6" t="s">
         <v>57</v>
       </c>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="4" t="s">
+      <c r="B20" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="6" t="s">
         <v>60</v>
       </c>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="4" t="s">
+      <c r="B21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="6" t="s">
         <v>64</v>
       </c>
+      <c r="F21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="B22" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F22" s="2"/>
+      <c r="F22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="B23" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F23" s="2"/>
+      <c r="F23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="B24" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="4" t="s">
+      <c r="B25" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="6" t="s">
         <v>78</v>
       </c>
+      <c r="F25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="4" t="s">
+      <c r="B26" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E26" s="4"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" s="4" t="s">
+      <c r="B27" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="6" t="s">
         <v>84</v>
       </c>
+      <c r="F27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C28" s="4" t="s">
+      <c r="B28" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="6" t="s">
         <v>88</v>
       </c>
+      <c r="F28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C29" s="4" t="s">
+      <c r="B29" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="6" t="s">
         <v>92</v>
       </c>
+      <c r="F29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="6" t="s">
         <v>94</v>
       </c>
+      <c r="D32" s="7" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B33" s="4" t="s">
+      <c r="A33" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>94</v>
       </c>
+      <c r="D33" s="6" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B34" s="4" t="s">
+      <c r="A34" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>94</v>
       </c>
+      <c r="D34" s="4" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>100</v>
+      <c r="A35" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>102</v>
+      <c r="A36" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>102</v>
+      <c r="A37" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>102</v>
+      <c r="A38" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>102</v>
+      <c r="A39" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Separate JSTV specific parts into separate class files for reuse
</commit_message>
<xml_diff>
--- a/Events.xlsx
+++ b/Events.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="113">
   <si>
     <t xml:space="preserve">Event Name</t>
   </si>
@@ -88,6 +88,9 @@
     <t xml:space="preserve">"destination_username":"alastar17"}</t>
   </si>
   <si>
+    <t xml:space="preserve">Raid In</t>
+  </si>
+  <si>
     <t xml:space="preserve">TipGoalDeleted</t>
   </si>
   <si>
@@ -194,6 +197,9 @@
   </si>
   <si>
     <t xml:space="preserve">"number_of_viewers":5}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raid Out?</t>
   </si>
   <si>
     <t xml:space="preserve">GiftedSubscriptions</t>
@@ -464,16 +470,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -497,7 +499,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -581,37 +583,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -684,7 +686,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.6"/>
@@ -706,85 +708,85 @@
       <c r="C1" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="n">
+      <c r="D1" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="n">
+      <c r="E1" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="n">
+      <c r="F1" s="2" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
@@ -803,458 +805,464 @@
         <v>21</v>
       </c>
       <c r="F7" s="6"/>
+      <c r="G7" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
+      <c r="C8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
+      <c r="C9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+      <c r="C10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="6" t="s">
+      <c r="A11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="C11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="6" t="s">
+      <c r="A12" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
+      <c r="C12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="6" t="s">
+      <c r="A13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="D13" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="6"/>
+      <c r="E13" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+      <c r="B14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
+      <c r="B15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="A16" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="B16" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="B17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="D17" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="4"/>
+      <c r="E17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" s="6" t="s">
+      <c r="A19" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="B19" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
+      <c r="D19" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="1" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D20" s="6" t="s">
+      <c r="A20" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
+      <c r="B20" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="A21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="B21" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="6"/>
+      <c r="D21" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F22" s="4"/>
+      <c r="B22" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E23" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F23" s="4"/>
+      <c r="B23" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="B24" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="F24" s="4" t="s">
-        <v>52</v>
+      <c r="D24" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="D25" s="6" t="s">
+      <c r="A25" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="B25" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="F25" s="6"/>
+      <c r="D25" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="F25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="6" t="s">
+      <c r="A26" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D26" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="D27" s="6" t="s">
+      <c r="A27" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="B27" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F27" s="6"/>
+      <c r="D27" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="D28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="B28" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F28" s="6"/>
+      <c r="D28" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="D29" s="6" t="s">
+      <c r="A29" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="B29" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F29" s="6"/>
+      <c r="D29" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>94</v>
+      <c r="A30" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>94</v>
+      <c r="A31" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B32" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>97</v>
+      <c r="D32" s="6" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>99</v>
+      <c r="A33" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>101</v>
+      <c r="A34" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="D35" s="8" t="s">
+      <c r="A35" s="5" t="s">
         <v>104</v>
       </c>
+      <c r="B35" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="D36" s="5" t="s">
+      <c r="A36" s="5" t="s">
         <v>107</v>
       </c>
+      <c r="B36" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>106</v>
-      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>106</v>
+      <c r="A38" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>106</v>
+      <c r="A39" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>